<commit_message>
remove the from the NMDP
</commit_message>
<xml_diff>
--- a/build/output/CodeSystem-cibmtr-ancestry-cs.xlsx
+++ b/build/output/CodeSystem-cibmtr-ancestry-cs.xlsx
@@ -57,19 +57,19 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-22T08:51:47-05:00</t>
+    <t>2026-06-22T09:21:59-05:00</t>
   </si>
   <si>
     <t>Publisher</t>
   </si>
   <si>
-    <t>The Medical College of Wisconsin, Inc. and the NMDP</t>
+    <t>The Medical College of Wisconsin, Inc. and NMDP</t>
   </si>
   <si>
     <t>Contact</t>
   </si>
   <si>
-    <t>The Medical College of Wisconsin, Inc. and the NMDP (http://www.cibmtr.org)</t>
+    <t>The Medical College of Wisconsin, Inc. and NMDP (http://www.cibmtr.org)</t>
   </si>
   <si>
     <t>Bob Milius (bmilius@nmdp.org)</t>

</xml_diff>